<commit_message>
chore: update sunday arrivals workbook
</commit_message>
<xml_diff>
--- a/Sunday_Arrivals.xlsx
+++ b/Sunday_Arrivals.xlsx
@@ -444,12 +444,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -483,10 +483,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D3" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -501,10 +501,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -519,10 +519,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -537,10 +537,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D6" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7">
@@ -550,10 +550,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>202</v>
+        <v>225</v>
       </c>
       <c r="D7" t="n">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
@@ -589,7 +589,7 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>154</v>
+        <v>120</v>
       </c>
       <c r="D11" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12">
@@ -622,10 +622,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
@@ -640,10 +640,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D13" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14">
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="D15" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
@@ -689,10 +689,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>486</v>
+        <v>413</v>
       </c>
       <c r="D16" t="n">
-        <v>413</v>
+        <v>396</v>
       </c>
     </row>
     <row r="18">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D18" t="n">
         <v>65</v>
@@ -725,10 +725,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>140</v>
+        <v>107</v>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20">
@@ -743,10 +743,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>125</v>
+        <v>47</v>
       </c>
       <c r="D20" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21">
@@ -756,10 +756,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>362</v>
+        <v>219</v>
       </c>
       <c r="D21" t="n">
-        <v>219</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23">
@@ -769,10 +769,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1050</v>
+        <v>857</v>
       </c>
       <c r="D23" t="n">
-        <v>857</v>
+        <v>846</v>
       </c>
     </row>
   </sheetData>
@@ -802,12 +802,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -859,10 +859,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -877,10 +877,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -913,10 +913,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -931,10 +931,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -949,10 +949,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -967,10 +967,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -985,10 +985,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D12" t="n">
         <v>8</v>
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="C13" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" t="n">
         <v>4</v>
-      </c>
-      <c r="D13" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D15" t="n">
         <v>65</v>
@@ -1085,12 +1085,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -1106,10 +1106,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D2" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -1142,10 +1142,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D5" t="n">
         <v>23</v>
@@ -1173,10 +1173,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D6" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1206,12 +1206,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -1248,7 +1248,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1281,10 +1281,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1320,7 +1320,7 @@
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1335,10 +1335,10 @@
         </is>
       </c>
       <c r="C8" t="n">
+        <v>22</v>
+      </c>
+      <c r="D8" t="n">
         <v>13</v>
-      </c>
-      <c r="D8" t="n">
-        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1353,10 +1353,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1371,10 +1371,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1389,10 +1389,10 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
         <v>5</v>
-      </c>
-      <c r="D11" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1407,10 +1407,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
@@ -1425,10 +1425,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1438,10 +1438,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D14" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1471,12 +1471,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -1492,10 +1492,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1510,10 +1510,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1528,10 +1528,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
@@ -1567,7 +1567,7 @@
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1582,10 +1582,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -1600,10 +1600,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1672,10 +1672,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1690,10 +1690,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1708,10 +1708,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -1726,10 +1726,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1762,10 +1762,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -1775,10 +1775,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>140</v>
+        <v>107</v>
       </c>
       <c r="D18" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1808,12 +1808,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -1847,10 +1847,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -1883,10 +1883,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -1904,7 +1904,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1919,10 +1919,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -1955,10 +1955,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -2027,10 +2027,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -2045,10 +2045,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -2063,10 +2063,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2081,10 +2081,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D16" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -2099,10 +2099,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2112,10 +2112,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>125</v>
+        <v>47</v>
       </c>
       <c r="D18" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2145,12 +2145,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -2166,10 +2166,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -2202,10 +2202,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -2223,7 +2223,7 @@
         <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -2238,10 +2238,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2256,10 +2256,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -2274,10 +2274,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -2292,10 +2292,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -2310,10 +2310,10 @@
         </is>
       </c>
       <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
         <v>6</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -2323,10 +2323,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2356,12 +2356,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
         <v>9</v>
@@ -2413,10 +2413,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -2431,10 +2431,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -2452,7 +2452,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
         <v>3</v>
@@ -2503,10 +2503,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -2557,10 +2557,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2570,10 +2570,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="D13" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2603,12 +2603,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -2624,10 +2624,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -2642,10 +2642,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2673,10 +2673,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D5" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2706,12 +2706,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -2745,10 +2745,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -2784,7 +2784,7 @@
         <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -2799,10 +2799,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -2838,7 +2838,7 @@
         <v>14</v>
       </c>
       <c r="D8" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -2853,10 +2853,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -2871,10 +2871,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -2902,10 +2902,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D12" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -2935,12 +2935,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -2992,10 +2992,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -3028,10 +3028,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -3046,10 +3046,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3059,10 +3059,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D8" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -3092,12 +3092,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -3113,10 +3113,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -3131,10 +3131,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -3149,10 +3149,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -3162,10 +3162,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3195,12 +3195,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -3216,10 +3216,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -3234,10 +3234,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -3252,10 +3252,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -3270,10 +3270,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -3288,10 +3288,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -3306,10 +3306,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -3337,10 +3337,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D9" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -3476,10 +3476,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -3492,7 +3492,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -3506,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3522,12 +3522,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>23/08</t>
+          <t>30/08</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>30/08</t>
+          <t>06/09</t>
         </is>
       </c>
     </row>
@@ -3543,185 +3543,167 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Adabraka</t>
+          <t>Arena</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Emmanuel Otiboe</t>
+          <t>Zephaniah Lartey</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arena</t>
+          <t>ATU Church</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Zephaniah Lartey</t>
+          <t>James Pekyie</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ATU Church</t>
+          <t>ATU Main Campus</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>James Pekyie</t>
+          <t>Racheal Boamah</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ATU Main Campus</t>
+          <t>City Campus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Racheal Boamah</t>
+          <t>Abednego Abbey</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>City Campus</t>
+          <t>Jamestown</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abednego Abbey</t>
+          <t>Joel Quartey</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jamestown</t>
+          <t>Jamestown Allos</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joel Quartey</t>
+          <t>Ishmael Oplerm</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jamestown Allos</t>
+          <t>UssherFort</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ishmael Oplerm</t>
+          <t>Seth Kpelebe</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UssherFort</t>
+          <t>Yours and Ours</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Seth Kpelebe</t>
+          <t>Prince Odum</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yours and Ours</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Prince Odum</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>120</v>
       </c>
       <c r="D11" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>154</v>
-      </c>
-      <c r="D12" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>